<commit_message>
Daily NSE scan: 2026-09-24
</commit_message>
<xml_diff>
--- a/output/2026-09-24/enriched_analysis.xlsx
+++ b/output/2026-09-24/enriched_analysis.xlsx
@@ -929,10 +929,10 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>3.578</v>
+        <v>3.577</v>
       </c>
       <c r="W2" t="n">
-        <v>2960</v>
+        <v>2961</v>
       </c>
       <c r="X2" t="n">
         <v>23.2</v>
@@ -1164,10 +1164,10 @@
         <v>0.051</v>
       </c>
       <c r="W3" t="n">
-        <v>2622</v>
+        <v>2627</v>
       </c>
       <c r="X3" t="n">
-        <v>9.01</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="Y3" t="n">
         <v>36</v>
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0.974</v>
+        <v>0.951</v>
       </c>
       <c r="W5" t="n">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="X5" t="n">
-        <v>8.77</v>
+        <v>8.98</v>
       </c>
       <c r="Y5" t="n">
         <v>17</v>
@@ -1861,7 +1861,7 @@
         <v>320</v>
       </c>
       <c r="X6" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="Y6" t="n">
         <v>22</v>
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.305</v>
+        <v>0.304</v>
       </c>
       <c r="W7" t="n">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="X7" t="n">
-        <v>9.869999999999999</v>
+        <v>9.92</v>
       </c>
       <c r="Y7" t="n">
         <v>7</v>
@@ -2786,7 +2786,7 @@
         <v>0.382</v>
       </c>
       <c r="W10" t="n">
-        <v>2724</v>
+        <v>2723</v>
       </c>
       <c r="X10" t="n">
         <v>22.3</v>
@@ -3018,10 +3018,10 @@
         <v>0.044</v>
       </c>
       <c r="W11" t="n">
-        <v>16488</v>
+        <v>16526</v>
       </c>
       <c r="X11" t="n">
-        <v>42</v>
+        <v>42.1</v>
       </c>
       <c r="Y11" t="n">
         <v>83</v>
@@ -3250,7 +3250,7 @@
         <v>0.397</v>
       </c>
       <c r="W12" t="n">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="X12" t="n">
         <v>60.2</v>
@@ -3479,10 +3479,10 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>1.572</v>
+        <v>1.585</v>
       </c>
       <c r="W13" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="n">
@@ -3709,13 +3709,13 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.163</v>
+        <v>0.159</v>
       </c>
       <c r="W14" t="n">
-        <v>678</v>
+        <v>698</v>
       </c>
       <c r="X14" t="n">
-        <v>56.7</v>
+        <v>58.3</v>
       </c>
       <c r="Y14" t="n">
         <v>3</v>
@@ -3941,13 +3941,13 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>2.306</v>
+        <v>2.288</v>
       </c>
       <c r="W15" t="n">
-        <v>2584</v>
+        <v>2604</v>
       </c>
       <c r="X15" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Y15" t="n">
         <v>6</v>
@@ -4176,10 +4176,10 @@
         <v>0.098</v>
       </c>
       <c r="W16" t="n">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="X16" t="n">
-        <v>28</v>
+        <v>27.9</v>
       </c>
       <c r="Y16" t="n">
         <v>24</v>
@@ -4637,10 +4637,10 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>2.823</v>
+        <v>2.827</v>
       </c>
       <c r="W18" t="n">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="X18" t="n">
         <v>26.2</v>
@@ -4866,7 +4866,7 @@
         <v>0.039</v>
       </c>
       <c r="W19" t="n">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="X19" t="n">
         <v>11.6</v>
@@ -5095,13 +5095,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.443</v>
+        <v>0.44</v>
       </c>
       <c r="W20" t="n">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="X20" t="n">
-        <v>38.9</v>
+        <v>39</v>
       </c>
       <c r="Y20" t="n">
         <v>21</v>
@@ -5330,10 +5330,10 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="W21" t="n">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="X21" t="n">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="Y21" t="n">
         <v>19</v>
@@ -5557,13 +5557,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.293</v>
+        <v>0.296</v>
       </c>
       <c r="W22" t="n">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="X22" t="n">
-        <v>25.3</v>
+        <v>24.9</v>
       </c>
       <c r="Y22" t="n">
         <v>12</v>
@@ -5792,10 +5792,10 @@
         <v>0.134</v>
       </c>
       <c r="W23" t="n">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="X23" t="n">
-        <v>5.98</v>
+        <v>5.99</v>
       </c>
       <c r="Y23" t="n">
         <v>118</v>
@@ -5808,7 +5808,7 @@
         <v>1.03</v>
       </c>
       <c r="AC23" t="n">
-        <v>18.5</v>
+        <v>19.9</v>
       </c>
       <c r="AD23" t="n">
         <v>0.01</v>
@@ -6255,7 +6255,7 @@
         <v>380</v>
       </c>
       <c r="X25" t="n">
-        <v>1225</v>
+        <v>1227</v>
       </c>
       <c r="Y25" t="n">
         <v>-61</v>
@@ -6480,7 +6480,7 @@
         <v>0.038</v>
       </c>
       <c r="W26" t="n">
-        <v>3567</v>
+        <v>3569</v>
       </c>
       <c r="X26" t="n">
         <v>21.2</v>
@@ -6712,7 +6712,7 @@
         <v>0.024</v>
       </c>
       <c r="W27" t="n">
-        <v>1029</v>
+        <v>1039</v>
       </c>
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="n">
@@ -7174,7 +7174,7 @@
         <v>0.052</v>
       </c>
       <c r="W29" t="n">
-        <v>5035</v>
+        <v>5036</v>
       </c>
       <c r="X29" t="n">
         <v>32.8</v>
@@ -7406,7 +7406,7 @@
         <v>0.057</v>
       </c>
       <c r="W30" t="n">
-        <v>1937</v>
+        <v>1940</v>
       </c>
       <c r="X30" t="n">
         <v>44.5</v>
@@ -7638,7 +7638,7 @@
         <v>0.514</v>
       </c>
       <c r="W31" t="n">
-        <v>3763</v>
+        <v>3764</v>
       </c>
       <c r="X31" t="n">
         <v>26.3</v>
@@ -7867,10 +7867,10 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.651</v>
+        <v>0.653</v>
       </c>
       <c r="W32" t="n">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="X32" t="n">
         <v>11.1</v>
@@ -8099,13 +8099,13 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.096</v>
+        <v>0.095</v>
       </c>
       <c r="W33" t="n">
-        <v>1553</v>
+        <v>1557</v>
       </c>
       <c r="X33" t="n">
-        <v>14</v>
+        <v>14.1</v>
       </c>
       <c r="Y33" t="n">
         <v>6</v>
@@ -8331,13 +8331,13 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="W34" t="n">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="X34" t="n">
-        <v>7.34</v>
+        <v>7.27</v>
       </c>
       <c r="Y34" t="n">
         <v>31</v>
@@ -9026,7 +9026,7 @@
         <v>0.021</v>
       </c>
       <c r="W37" t="n">
-        <v>9407</v>
+        <v>9416</v>
       </c>
       <c r="X37" t="n">
         <v>12.4</v>
@@ -9258,10 +9258,10 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>3859</v>
+        <v>3849</v>
       </c>
       <c r="X38" t="n">
-        <v>86.90000000000001</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="Y38" t="n">
         <v>42</v>
@@ -9954,10 +9954,10 @@
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="X41" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="Y41" t="n">
         <v>5</v>
@@ -10183,13 +10183,13 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>0.127</v>
+        <v>0.128</v>
       </c>
       <c r="W42" t="n">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="X42" t="n">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="Y42" t="n">
         <v>61</v>
@@ -10413,13 +10413,13 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.291</v>
+        <v>0.294</v>
       </c>
       <c r="W43" t="n">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="X43" t="n">
-        <v>15.2</v>
+        <v>15</v>
       </c>
       <c r="Y43" t="n">
         <v>16</v>
@@ -10645,13 +10645,13 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.228</v>
+        <v>0.227</v>
       </c>
       <c r="W44" t="n">
-        <v>989</v>
+        <v>992</v>
       </c>
       <c r="X44" t="n">
-        <v>26.9</v>
+        <v>27</v>
       </c>
       <c r="Y44" t="n">
         <v>9</v>
@@ -11342,7 +11342,7 @@
         <v>0</v>
       </c>
       <c r="W47" t="n">
-        <v>9131</v>
+        <v>9142</v>
       </c>
       <c r="X47" t="n">
         <v>15.5</v>
@@ -11574,10 +11574,10 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>120154</v>
+        <v>119891</v>
       </c>
       <c r="X48" t="n">
-        <v>34.6</v>
+        <v>34.5</v>
       </c>
       <c r="Y48" t="n">
         <v>18</v>
@@ -12035,13 +12035,13 @@
         </is>
       </c>
       <c r="V50" t="n">
-        <v>0.351</v>
+        <v>0.35</v>
       </c>
       <c r="W50" t="n">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="X50" t="n">
-        <v>98.7</v>
+        <v>99</v>
       </c>
       <c r="Y50" t="n">
         <v>246</v>
@@ -12270,7 +12270,7 @@
         <v>0.042</v>
       </c>
       <c r="W51" t="n">
-        <v>1635</v>
+        <v>1636</v>
       </c>
       <c r="X51" t="n">
         <v>21.4</v>
@@ -12502,7 +12502,7 @@
         <v>0.081</v>
       </c>
       <c r="W52" t="n">
-        <v>1688</v>
+        <v>1690</v>
       </c>
       <c r="X52" t="n">
         <v>30.5</v>

</xml_diff>